<commit_message>
initial tables for new modules
</commit_message>
<xml_diff>
--- a/data/projects.xlsx
+++ b/data/projects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aheller\Documents\GitHub\TEA.CART\inst\app\www\static_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camsys-my.sharepoint.com/personal/slarue_camsys_com/Documents/Documents/idot_github_puller/TEACART/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52EA532E-CF08-4F00-9C00-405B04748FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{52EA532E-CF08-4F00-9C00-405B04748FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A260C76-F02B-477D-84D8-9803BCEFCF51}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{CAB68D25-6356-4621-A47F-2914E781935C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="10" activeTab="15" xr2:uid="{CAB68D25-6356-4621-A47F-2914E781935C}"/>
   </bookViews>
   <sheets>
     <sheet name="bikeped" sheetId="1" r:id="rId1"/>
@@ -27,6 +27,9 @@
     <sheet name="evsi" sheetId="12" r:id="rId12"/>
     <sheet name="freight" sheetId="13" r:id="rId13"/>
     <sheet name="expansion" sheetId="14" r:id="rId14"/>
+    <sheet name="transit_cuts" sheetId="15" r:id="rId15"/>
+    <sheet name="land_use" sheetId="16" r:id="rId16"/>
+    <sheet name="road_resurf" sheetId="17" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="102">
   <si>
     <t>Bicycle and Pedestrian</t>
   </si>
@@ -307,6 +310,54 @@
   </si>
   <si>
     <t>Arterial</t>
+  </si>
+  <si>
+    <t>Service Type</t>
+  </si>
+  <si>
+    <t>Fixed Route Bus</t>
+  </si>
+  <si>
+    <t>Demand Response</t>
+  </si>
+  <si>
+    <t>Light Rail</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Transit Service Cuts</t>
+  </si>
+  <si>
+    <t>#removed voms</t>
+  </si>
+  <si>
+    <t>Land Use</t>
+  </si>
+  <si>
+    <t>#units</t>
+  </si>
+  <si>
+    <t>Land Use Incentives</t>
+  </si>
+  <si>
+    <t>$million</t>
+  </si>
+  <si>
+    <t>Increase Residential Density</t>
+  </si>
+  <si>
+    <t># rezoned acres</t>
+  </si>
+  <si>
+    <t>Increase Job Density</t>
+  </si>
+  <si>
+    <t>Mixed-Use TOD (higher intensity)</t>
+  </si>
+  <si>
+    <t>Mixed-Use TOD (moderate intensity)</t>
   </si>
 </sst>
 </file>
@@ -362,9 +413,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -402,7 +453,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -508,7 +559,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -650,7 +701,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -659,9 +710,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C95435C7-2DE4-48D1-9E53-4031801771FF}">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -669,7 +720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -686,7 +737,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -694,7 +745,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -702,7 +753,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -710,7 +761,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -718,7 +769,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -726,7 +777,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -734,7 +785,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -742,7 +793,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -750,7 +801,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -758,7 +809,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -766,7 +817,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -774,7 +825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -782,7 +833,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -790,7 +841,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -798,7 +849,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -806,7 +857,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -814,7 +865,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -822,7 +873,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -830,7 +881,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -838,7 +889,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -846,7 +897,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -862,9 +913,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAD35E33-7FCE-4DAE-ADE3-B97F83018830}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>60</v>
       </c>
@@ -872,7 +923,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>61</v>
       </c>
@@ -889,7 +940,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>63</v>
       </c>
@@ -897,7 +948,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -905,7 +956,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>65</v>
       </c>
@@ -913,7 +964,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>66</v>
       </c>
@@ -921,7 +972,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>67</v>
       </c>
@@ -937,9 +988,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D937B4B-0BBE-42AF-A39C-1FA5C009FAE0}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -947,7 +998,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -964,7 +1015,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -980,9 +1031,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F63B95A-05A5-4E83-8CEE-BE78DB93017B}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>71</v>
       </c>
@@ -990,7 +1041,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>72</v>
       </c>
@@ -1007,7 +1058,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -1015,7 +1066,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -1023,7 +1074,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>76</v>
       </c>
@@ -1031,7 +1082,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>77</v>
       </c>
@@ -1039,7 +1090,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>78</v>
       </c>
@@ -1055,9 +1106,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45C80BBC-96E9-4DD5-9EC6-D6E4E814D9D9}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>79</v>
       </c>
@@ -1065,7 +1116,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>80</v>
       </c>
@@ -1082,7 +1133,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -1098,9 +1149,12 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3782BC60-4233-4F37-9FFA-69AE58DFF358}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>82</v>
       </c>
@@ -1108,7 +1162,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1125,7 +1179,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>84</v>
       </c>
@@ -1133,7 +1187,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>84</v>
       </c>
@@ -1141,7 +1195,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>85</v>
       </c>
@@ -1149,7 +1203,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1162,85 +1216,93 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E62025BA-384B-4B5B-89DF-4F5D206F709F}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE2D9754-A3FC-43F6-A99C-9FD8241844C7}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="39.85546875" customWidth="1"/>
+    <col min="1" max="1" width="16.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>91</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>86</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2">
-        <v>2025</v>
+        <v>2030</v>
       </c>
       <c r="D2">
-        <v>2030</v>
+        <v>2040</v>
       </c>
       <c r="E2">
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1248,88 +1310,77 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D4E8BF9-53F0-496D-BD3B-B84D01811916}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD8BEB19-39E7-430B-AFDE-001EEB795690}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="41.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>93</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C2">
-        <v>2025</v>
+        <v>2030</v>
       </c>
       <c r="D2">
-        <v>2030</v>
+        <v>2040</v>
       </c>
       <c r="E2">
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1337,28 +1388,34 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10292699-683D-473D-A0CC-19422A51AA6F}">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48813ADD-5965-4508-A7D2-D748617066E7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E62025BA-384B-4B5B-89DF-4F5D206F709F}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1373,7 +1430,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1381,7 +1438,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1389,7 +1446,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1397,7 +1454,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1405,35 +1462,19 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1442,25 +1483,31 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94076854-7526-4AF0-AC6C-7C8FCD4A4BEF}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D4E8BF9-53F0-496D-BD3B-B84D01811916}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="41.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.1796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="C2">
         <v>2025</v>
@@ -1472,12 +1519,52 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1485,25 +1572,31 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3693B71-A429-47AD-8FFC-8C853E66C168}">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10292699-683D-473D-A0CC-19422A51AA6F}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="5.1796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="C2">
         <v>2025</v>
@@ -1515,36 +1608,68 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1552,22 +1677,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77677232-3C99-421C-A7BD-1765C48804EC}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94076854-7526-4AF0-AC6C-7C8FCD4A4BEF}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
         <v>32</v>
@@ -1582,12 +1707,12 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1595,25 +1720,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42345BAD-9809-444E-99A8-E50E4360BF2B}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3693B71-A429-47AD-8FFC-8C853E66C168}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C2">
         <v>2025</v>
@@ -1625,12 +1750,36 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1638,12 +1787,98 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77677232-3C99-421C-A7BD-1765C48804EC}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2">
+        <v>2025</v>
+      </c>
+      <c r="D2">
+        <v>2030</v>
+      </c>
+      <c r="E2">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42345BAD-9809-444E-99A8-E50E4360BF2B}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2">
+        <v>2025</v>
+      </c>
+      <c r="D2">
+        <v>2030</v>
+      </c>
+      <c r="E2">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9F8CBD9-CAFE-4076-810C-99408B15DCA5}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -1651,7 +1886,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>53</v>
       </c>
@@ -1668,7 +1903,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>55</v>
       </c>
@@ -1676,7 +1911,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>55</v>
       </c>
@@ -1684,7 +1919,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>58</v>
       </c>
@@ -1692,7 +1927,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>59</v>
       </c>

</xml_diff>